<commit_message>
479 préparation publication release 240 ballot (#486)
* release 240-ballot

* Update changes.md bc64af928b17ce000f3f84fb20700905397404d0
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-tddui-basic-decision-identifier.xlsx
+++ b/main/ig/CodeSystem-tddui-basic-decision-identifier.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.3.0</t>
+    <t>2.4.0-ballot</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-30T13:41:45+00:00</t>
+    <t>2026-06-30T14:01:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Publication finale de la release 2.4.0 (#498)
* Publi 240

* trial use 131adca4787997b63c58cf23e271f2e7de064117
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-tddui-basic-decision-identifier.xlsx
+++ b/main/ig/CodeSystem-tddui-basic-decision-identifier.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.4.0-ballot</t>
+    <t>2.4.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-20T07:42:46+00:00</t>
+    <t>2026-07-22T13:04:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>